<commit_message>
@ fix: sheet DiscreteAnalog saia com linha-fantasma do template
- pre-limpa sheets de sinais sem dados no import (remove leftover)
- limpa valores da linha-template da DA no reference_template.xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/backend/data/reference_template.xlsx
+++ b/backend/data/reference_template.xlsx
@@ -18166,7 +18166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV5"/>
+  <dimension ref="A1:BI5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="24.140625" customWidth="1" style="19" min="1" max="1"/>
@@ -18260,11 +18260,7 @@
       <c r="U1" s="20" t="n"/>
       <c r="V1" s="20" t="n"/>
       <c r="W1" s="20" t="n"/>
-      <c r="X1" s="20" t="inlineStr">
-        <is>
-          <t>Remote Points</t>
-        </is>
-      </c>
+      <c r="X1" s="20" t="n"/>
       <c r="Y1" s="20" t="n"/>
       <c r="Z1" s="20" t="n"/>
       <c r="AA1" s="20" t="n"/>
@@ -18293,6 +18289,19 @@
       <c r="AT1" s="20" t="n"/>
       <c r="AU1" s="20" t="n"/>
       <c r="AV1" s="20" t="n"/>
+      <c r="AW1" s="20" t="n"/>
+      <c r="AX1" s="20" t="n"/>
+      <c r="AY1" s="20" t="n"/>
+      <c r="AZ1" s="20" t="n"/>
+      <c r="BA1" s="20" t="n"/>
+      <c r="BB1" s="20" t="n"/>
+      <c r="BC1" s="20" t="n"/>
+      <c r="BD1" s="20" t="n"/>
+      <c r="BE1" s="20" t="n"/>
+      <c r="BF1" s="20" t="n"/>
+      <c r="BG1" s="20" t="n"/>
+      <c r="BH1" s="20" t="n"/>
+      <c r="BI1" s="21" t="n"/>
     </row>
     <row r="2" hidden="1" ht="18" customHeight="1" s="19">
       <c r="A2" s="12" t="inlineStr">
@@ -18322,11 +18331,7 @@
       <c r="U2" s="20" t="n"/>
       <c r="V2" s="20" t="n"/>
       <c r="W2" s="20" t="n"/>
-      <c r="X2" s="20" t="inlineStr">
-        <is>
-          <t>REMOTEPOINT</t>
-        </is>
-      </c>
+      <c r="X2" s="20" t="n"/>
       <c r="Y2" s="20" t="n"/>
       <c r="Z2" s="20" t="n"/>
       <c r="AA2" s="21" t="n"/>
@@ -18352,17 +18357,19 @@
       <c r="AM2" s="20" t="n"/>
       <c r="AN2" s="20" t="n"/>
       <c r="AO2" s="20" t="n"/>
-      <c r="AP2" s="20" t="inlineStr">
-        <is>
-          <t>APROCESSING</t>
-        </is>
-      </c>
+      <c r="AP2" s="20" t="n"/>
       <c r="AQ2" s="20" t="n"/>
       <c r="AR2" s="20" t="n"/>
       <c r="AS2" s="20" t="n"/>
       <c r="AT2" s="20" t="n"/>
       <c r="AU2" s="20" t="n"/>
       <c r="AV2" s="20" t="n"/>
+      <c r="AW2" s="20" t="n"/>
+      <c r="AX2" s="20" t="n"/>
+      <c r="AY2" s="20" t="n"/>
+      <c r="AZ2" s="20" t="n"/>
+      <c r="BA2" s="20" t="n"/>
+      <c r="BB2" s="21" t="n"/>
     </row>
     <row r="3" hidden="1" ht="18" customHeight="1" s="19">
       <c r="A3" s="12" t="inlineStr">
@@ -18821,132 +18828,51 @@
       </c>
     </row>
     <row r="5" ht="18" customHeight="1" s="19">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>FWB_AL13_52-13_IA</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr"/>
-      <c r="C5" s="18" t="inlineStr">
-        <is>
-          <t>IA</t>
-        </is>
-      </c>
-      <c r="E5" s="18" t="inlineStr">
-        <is>
-          <t>Current</t>
-        </is>
-      </c>
-      <c r="F5" s="18" t="inlineStr">
-        <is>
-          <t>SCD Distr</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="inlineStr"/>
-      <c r="H5" s="18" t="inlineStr"/>
-      <c r="I5" s="18" t="inlineStr"/>
-      <c r="J5" s="18" t="inlineStr"/>
-      <c r="K5" s="18" t="inlineStr"/>
-      <c r="L5" s="18" t="inlineStr"/>
-      <c r="M5" s="18" t="inlineStr">
-        <is>
-          <t>FWB_AL13_52-13_DJ</t>
-        </is>
-      </c>
-      <c r="N5" s="18" t="inlineStr"/>
-      <c r="O5" s="18" t="inlineStr">
-        <is>
-          <t>MeasuredValue</t>
-        </is>
-      </c>
-      <c r="P5" s="18" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="Q5" s="18" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="R5" s="18" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="S5" s="18" t="inlineStr">
-        <is>
-          <t>Read</t>
-        </is>
-      </c>
-      <c r="T5" s="18" t="inlineStr"/>
-      <c r="U5" s="18" t="inlineStr">
-        <is>
-          <t>Undirected</t>
-        </is>
-      </c>
-      <c r="V5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" s="18" t="n">
-        <v>100</v>
-      </c>
-      <c r="Y5" s="18" t="n">
-        <v>-1</v>
-      </c>
-      <c r="Z5" s="18" t="inlineStr">
-        <is>
-          <t>I_403.2@null_null@null_Distr</t>
-        </is>
-      </c>
-      <c r="AA5" s="18" t="inlineStr">
-        <is>
-          <t>UTR_FWB_1</t>
-        </is>
-      </c>
-      <c r="AB5" s="18" t="inlineStr"/>
-      <c r="AC5" s="18" t="inlineStr"/>
-      <c r="AD5" s="18" t="inlineStr"/>
-      <c r="AE5" s="18" t="inlineStr"/>
-      <c r="AF5" s="18" t="inlineStr"/>
-      <c r="AG5" s="18" t="inlineStr"/>
-      <c r="AH5" s="18" t="inlineStr"/>
-      <c r="AI5" s="18" t="inlineStr"/>
-      <c r="AJ5" s="18" t="inlineStr"/>
-      <c r="AK5" s="18">
-        <f>DNP3_AnalogSignals[[#This Row],[Signal Name]]</f>
-        <v/>
-      </c>
-      <c r="AL5" s="18" t="inlineStr"/>
-      <c r="AM5" s="18" t="inlineStr">
-        <is>
-          <t>FWB_AS_00062</t>
-        </is>
-      </c>
-      <c r="AN5" s="18" t="n">
-        <v>20260416</v>
-      </c>
-      <c r="AO5" s="18" t="inlineStr">
-        <is>
-          <t>Analog</t>
-        </is>
-      </c>
-      <c r="AP5" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="AT5" s="18" t="inlineStr"/>
-      <c r="AV5" s="18" t="n">
-        <v>41</v>
-      </c>
+      <c r="A5" s="18" t="n"/>
+      <c r="B5" s="18" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="18" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="n"/>
+      <c r="R5" s="18" t="n"/>
+      <c r="S5" s="18" t="n"/>
+      <c r="T5" s="18" t="n"/>
+      <c r="U5" s="18" t="n"/>
+      <c r="V5" s="18" t="n"/>
+      <c r="W5" s="18" t="n"/>
+      <c r="X5" s="18" t="n"/>
+      <c r="Y5" s="18" t="n"/>
+      <c r="Z5" s="18" t="n"/>
+      <c r="AA5" s="18" t="n"/>
+      <c r="AB5" s="18" t="n"/>
+      <c r="AC5" s="18" t="n"/>
+      <c r="AD5" s="18" t="n"/>
+      <c r="AE5" s="18" t="n"/>
+      <c r="AF5" s="18" t="n"/>
+      <c r="AG5" s="18" t="n"/>
+      <c r="AH5" s="18" t="n"/>
+      <c r="AI5" s="18" t="n"/>
+      <c r="AJ5" s="18" t="n"/>
+      <c r="AK5" s="18" t="n"/>
+      <c r="AL5" s="18" t="n"/>
+      <c r="AM5" s="18" t="n"/>
+      <c r="AN5" s="18" t="n"/>
+      <c r="AO5" s="18" t="n"/>
+      <c r="AP5" s="18" t="n"/>
+      <c r="AQ5" s="18" t="n"/>
+      <c r="AR5" s="18" t="n"/>
+      <c r="AT5" s="18" t="n"/>
+      <c r="AV5" s="18" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="19"/>
     <row r="7" ht="18" customHeight="1" s="19"/>

</xml_diff>